<commit_message>
fixed bank account logic
</commit_message>
<xml_diff>
--- a/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
+++ b/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
@@ -2,20 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bank-account-monitoring\bams-backend\app\ds\llm\utils\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91977\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAC0E15-B112-4517-8DE4-55A178C4889A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D84B305-DB73-4501-A1C8-6AB733D2E4A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="8880" xr2:uid="{C9023426-1A3B-F741-8689-92A4FE46535A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C9023426-1A3B-F741-8689-92A4FE46535A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$46</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +30,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -37,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="85">
   <si>
     <t>S No</t>
   </si>
@@ -57,12 +62,6 @@
     <t>Email ID</t>
   </si>
   <si>
-    <t>R N Gupta</t>
-  </si>
-  <si>
-    <t>SBPRV</t>
-  </si>
-  <si>
     <t>maxwelldelhi</t>
   </si>
   <si>
@@ -72,9 +71,6 @@
     <t>Om Prakash Gupta</t>
   </si>
   <si>
-    <t>SBSPA</t>
-  </si>
-  <si>
     <t>OM Prakash Gupta HUF</t>
   </si>
   <si>
@@ -84,9 +80,6 @@
     <t>Ujjwal Gupta</t>
   </si>
   <si>
-    <t>SBEZY</t>
-  </si>
-  <si>
     <t>Ujjwal Gupta HUF</t>
   </si>
   <si>
@@ -102,21 +95,12 @@
     <t>Samriddhi Gupta</t>
   </si>
   <si>
-    <t>SBSPL</t>
-  </si>
-  <si>
     <t>gupta.samriddhi</t>
   </si>
   <si>
     <t>Umang Gupta</t>
   </si>
   <si>
-    <t>Umang Gupta NRE A/c</t>
-  </si>
-  <si>
-    <t>NRE A/c</t>
-  </si>
-  <si>
     <t>Vaibhav Gupta</t>
   </si>
   <si>
@@ -141,9 +125,6 @@
     <t>Umang Gupta NRE</t>
   </si>
   <si>
-    <t>Arvind Gupta</t>
-  </si>
-  <si>
     <t>478010100035662</t>
   </si>
   <si>
@@ -168,9 +149,6 @@
     <t>921010014965532</t>
   </si>
   <si>
-    <t>Arvind Kumar  Gupta</t>
-  </si>
-  <si>
     <t>478010100037989</t>
   </si>
   <si>
@@ -234,15 +212,9 @@
     <t>015501029775</t>
   </si>
   <si>
-    <t>SAAQB25K</t>
-  </si>
-  <si>
     <t>Maxwelldelhi</t>
   </si>
   <si>
-    <t>Arivind Gupta HUF</t>
-  </si>
-  <si>
     <t>Arvind Gupta Oorja/UG</t>
   </si>
   <si>
@@ -279,7 +251,52 @@
     <t>HDFC Bank</t>
   </si>
   <si>
-    <t>R N Gupta HUF</t>
+    <t xml:space="preserve">Umang Gupta NRE </t>
+  </si>
+  <si>
+    <t>UMANG  NRO</t>
+  </si>
+  <si>
+    <t>UMANG NRE</t>
+  </si>
+  <si>
+    <t>50100494729252</t>
+  </si>
+  <si>
+    <t>59108826833384</t>
+  </si>
+  <si>
+    <t>Bank of Baroda</t>
+  </si>
+  <si>
+    <t>12990100000673</t>
+  </si>
+  <si>
+    <t>Indusind Bank</t>
+  </si>
+  <si>
+    <t>159871207208</t>
+  </si>
+  <si>
+    <t>159311207208</t>
+  </si>
+  <si>
+    <t>159871897208</t>
+  </si>
+  <si>
+    <t>918800522020</t>
+  </si>
+  <si>
+    <t>State Bank of India</t>
+  </si>
+  <si>
+    <t>10591678294</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>NRE</t>
   </si>
 </sst>
 </file>
@@ -347,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -355,9 +372,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -692,11 +708,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F5EBB1F-53CB-2547-B69C-9927543A394B}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="19.09765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.296875" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.19921875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.69921875" bestFit="1" customWidth="1"/>
   </cols>
@@ -723,524 +740,552 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>35</v>
+        <v>83</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>36</v>
+        <v>83</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="E3" s="2">
         <v>9625340106</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>37</v>
+        <v>83</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="E4" s="2">
         <v>9625340106</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>38</v>
+        <v>83</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="E5" s="2">
         <v>9560255055</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>39</v>
+        <v>83</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="E6" s="2">
         <v>9871207208</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>40</v>
+        <v>83</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="E7" s="2">
         <v>9871207208</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>41</v>
+        <v>83</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="E8" s="2">
         <v>9953595755</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="7" t="s">
-        <v>42</v>
+        <v>12</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="E9" s="2">
         <v>9953595755</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>44</v>
+        <v>83</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="E10" s="2">
         <v>9871207208</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>45</v>
+        <v>83</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="E11" s="2">
         <v>9871207208</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>46</v>
+        <v>83</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="E12" s="2">
         <v>9871207208</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>47</v>
+        <v>83</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E13" s="2">
         <v>9871897208</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>48</v>
+        <v>83</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="E14" s="2">
         <v>9871207208</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>49</v>
+        <v>84</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="E15" s="2">
         <v>9871207208</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>50</v>
+        <v>83</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="E16" s="2">
         <v>925340106</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="D17" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="E17" s="5">
-        <v>9625340106</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+        <v>21</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="5">
+        <v>9625340106</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E19" s="5">
-        <v>9871207208</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="8" t="s">
-        <v>54</v>
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="E20" s="5">
-        <v>9560255055</v>
+        <v>9871207208</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+        <v>8</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="5">
+        <v>9560255055</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E22" s="5">
-        <v>9311107208</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="8" t="s">
-        <v>57</v>
+        <v>10</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="E23" s="5">
-        <v>9953595755</v>
+        <v>9311107208</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="5">
+        <v>9953595755</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E25" s="5">
-        <v>9871207208</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="5">
+        <v>9871207208</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="5">
-        <v>9311207208</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>8</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="8" t="s">
-        <v>62</v>
+        <v>15</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="E28" s="5">
-        <v>8800522020</v>
+        <v>9311207208</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="8" t="s">
-        <v>63</v>
+        <v>19</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="E29" s="5">
-        <v>9953595755</v>
-      </c>
-      <c r="F29" s="2"/>
+        <v>8800522020</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="8" t="s">
-        <v>64</v>
+        <v>25</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="E30" s="5">
         <v>9953595755</v>
@@ -1248,161 +1293,291 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="A31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="5">
+        <v>9953595755</v>
+      </c>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32" s="5"/>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E33" s="5"/>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B31" t="s">
+      <c r="E34" s="5"/>
+      <c r="F34" s="2"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E35" s="5"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E36" s="5"/>
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" s="2">
+        <v>9311207208</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E39" s="2">
+        <v>8851100933</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E40" s="2">
+        <v>9871207208</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E41" s="2">
+        <v>9871207208</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E42" s="2">
+        <v>9871207208</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E43" s="2">
+        <v>9953595755</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E31">
-        <v>9311207208</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="E44" s="2">
+        <v>9560255055</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E32">
-        <v>8851100933</v>
-      </c>
-      <c r="F32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>79</v>
-      </c>
-      <c r="B33" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E33">
-        <v>9871207208</v>
-      </c>
-      <c r="F33" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>79</v>
-      </c>
-      <c r="B34" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="E34">
-        <v>9871207208</v>
-      </c>
-      <c r="F34" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35" t="s">
-        <v>68</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E35">
-        <v>9871207208</v>
-      </c>
-      <c r="F35" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>79</v>
-      </c>
-      <c r="B36" t="s">
+      <c r="E45" s="2">
+        <v>9311107208</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C36" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="E36">
-        <v>9953595755</v>
-      </c>
-      <c r="F36" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>79</v>
-      </c>
-      <c r="B37" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E37">
-        <v>9560255055</v>
-      </c>
-      <c r="F37" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" t="s">
-        <v>13</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E38">
-        <v>9311107208</v>
-      </c>
-      <c r="F38" t="s">
-        <v>66</v>
+      <c r="C46" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working statement fetching from gmail
</commit_message>
<xml_diff>
--- a/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
+++ b/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C7E78C-E5A1-46DE-88E3-F3C15C28ECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="62">
   <si>
     <t>S No</t>
   </si>
@@ -35,6 +31,9 @@
     <t>Email ID</t>
   </si>
   <si>
+    <t>Password</t>
+  </si>
+  <si>
     <t>Axis Bank</t>
   </si>
   <si>
@@ -44,51 +43,90 @@
     <t>Savings</t>
   </si>
   <si>
+    <t>RAMN1006</t>
+  </si>
+  <si>
     <t>Ram Niwas Gupta HUF</t>
   </si>
   <si>
     <t>maxwelldelhi</t>
   </si>
   <si>
+    <t>RAMN478004897</t>
+  </si>
+  <si>
     <t>Bhagwati Devi</t>
   </si>
   <si>
+    <t>BHAG478004631</t>
+  </si>
+  <si>
     <t>Om Prakash Gupta</t>
   </si>
   <si>
+    <t>OMPR478004812</t>
+  </si>
+  <si>
     <t>OM Prakash Gupta HUF</t>
   </si>
   <si>
+    <t>OMPR478004952</t>
+  </si>
+  <si>
     <t>Sunita Gupta</t>
   </si>
   <si>
+    <t>SUNI478004689</t>
+  </si>
+  <si>
     <t>Ujjwal Gupta</t>
   </si>
   <si>
+    <t>UJJW478004632</t>
+  </si>
+  <si>
     <t>Ujjwal Gupta HUF</t>
   </si>
   <si>
     <t>ujjwal.gtd@g</t>
   </si>
   <si>
+    <t>UJJW905681456</t>
+  </si>
+  <si>
     <t>Arvind Kumar Gupta</t>
   </si>
   <si>
+    <t>ARVI478004879</t>
+  </si>
+  <si>
     <t>Arvind Kumar Gupta HUF</t>
   </si>
   <si>
+    <t>ARVI478004895</t>
+  </si>
+  <si>
     <t>Deepali Gupta</t>
   </si>
   <si>
+    <t>DEEP478004628</t>
+  </si>
+  <si>
     <t>Samriddhi Gupta</t>
   </si>
   <si>
     <t>gupta.samriddhi</t>
   </si>
   <si>
+    <t>SAMR3105</t>
+  </si>
+  <si>
     <t>Umang Gupta</t>
   </si>
   <si>
+    <t>UMAN2710</t>
+  </si>
+  <si>
     <t xml:space="preserve">Umang Gupta NRE </t>
   </si>
   <si>
@@ -98,6 +136,9 @@
     <t>Vaibhav Gupta</t>
   </si>
   <si>
+    <t>VAIB478005339</t>
+  </si>
+  <si>
     <t>Bank of Baroda</t>
   </si>
   <si>
@@ -116,12 +157,24 @@
     <t>Indusind Bank</t>
   </si>
   <si>
+    <t>ARVI0311</t>
+  </si>
+  <si>
+    <t>DEEP2811</t>
+  </si>
+  <si>
+    <t>VAIB2312</t>
+  </si>
+  <si>
     <t>HDFC Bank</t>
   </si>
   <si>
     <t>UMANG  NRO</t>
   </si>
   <si>
+    <t>NOT ACTIVE</t>
+  </si>
+  <si>
     <t>UMANG NRE</t>
   </si>
   <si>
@@ -143,59 +196,20 @@
     <t>CURRENT ACCOUNT FOR MCA</t>
   </si>
   <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>RAMN1006</t>
-  </si>
-  <si>
-    <t>BHAG2808</t>
-  </si>
-  <si>
-    <t>OMPR1811</t>
-  </si>
-  <si>
-    <t>UJJW0405</t>
-  </si>
-  <si>
-    <t>ARVI0311</t>
-  </si>
-  <si>
-    <t>DEEP2811</t>
-  </si>
-  <si>
-    <t>SAMR3105</t>
-  </si>
-  <si>
-    <t>UMAN2710</t>
-  </si>
-  <si>
-    <t>VAIB2312</t>
-  </si>
-  <si>
-    <t>ARVI2907</t>
-  </si>
-  <si>
-    <t>UJJW2003</t>
-  </si>
-  <si>
-    <t>SUNI0406</t>
-  </si>
-  <si>
-    <t>NOT ACTIVE</t>
+    <t>MODE478003676</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -208,38 +222,19 @@
     </font>
     <font>
       <u/>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FF333333"/>
       <sz val="11"/>
-      <color rgb="FF333333"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -259,16 +254,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
+      <left style="dotted">
         <color rgb="FF000000"/>
       </left>
-      <right style="hair">
+      <right style="dotted">
         <color rgb="FF000000"/>
       </right>
-      <top style="hair">
+      <top style="dotted">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="hair">
+      <bottom style="dotted">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
@@ -277,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -285,12 +280,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -631,21 +624,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="21.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="1" max="1" width="21.142857142857142" customWidth="1"/>
+    <col min="2" max="2" width="24.571428571428573" customWidth="1"/>
+    <col min="3" max="3" width="13.571428571428571" customWidth="1"/>
+    <col min="4" max="4" width="34.142857142857146" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625"/>
-    <col min="8" max="24" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="17.714285714285715" customWidth="1"/>
+    <col min="7" max="7" width="28.714285714285715" customWidth="1"/>
+    <col min="8" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -664,38 +657,38 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3">
         <v>478010100035662</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
-      <c r="G2" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3">
         <v>915010047947775</v>
@@ -704,21 +697,21 @@
         <v>9625340106</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3">
         <v>478010100035671</v>
@@ -727,21 +720,21 @@
         <v>9625340106</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3">
         <v>914010056197393</v>
@@ -750,21 +743,21 @@
         <v>9560255055</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3">
         <v>915010047121834</v>
@@ -773,21 +766,21 @@
         <v>9871207208</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3">
         <v>478010100036193</v>
@@ -796,21 +789,21 @@
         <v>9871207208</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3">
         <v>914010052112006</v>
@@ -819,21 +812,21 @@
         <v>9953595755</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="3">
         <v>921010014965532</v>
@@ -842,21 +835,21 @@
         <v>9953595755</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3">
         <v>478010100037989</v>
@@ -865,21 +858,21 @@
         <v>9871207208</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="3">
         <v>915010048076744</v>
@@ -888,21 +881,21 @@
         <v>9871207208</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3">
         <v>478010100035644</v>
@@ -911,21 +904,21 @@
         <v>9871207208</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" s="3">
         <v>478010100041450</v>
@@ -934,21 +927,21 @@
         <v>9871897208</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3">
         <v>478010100041618</v>
@@ -957,21 +950,21 @@
         <v>9871207208</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D15" s="3">
         <v>922010005537701</v>
@@ -980,21 +973,21 @@
         <v>9871207208</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" s="3">
         <v>915010023872994</v>
@@ -1003,21 +996,21 @@
         <v>925340106</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3">
         <v>12990100000673</v>
@@ -1025,15 +1018,15 @@
       <c r="E17" s="3"/>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D18" s="3">
         <v>15501544782</v>
@@ -1042,21 +1035,21 @@
         <v>9625340106</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="9">
+        <v>12</v>
+      </c>
+      <c r="G18" s="7">
         <v>590479799</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D19" s="3">
         <v>15501029814</v>
@@ -1064,15 +1057,15 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D20" s="3">
         <v>15501544789</v>
@@ -1081,21 +1074,21 @@
         <v>9871207208</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="9">
+        <v>12</v>
+      </c>
+      <c r="G20" s="7">
         <v>590479943</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D21" s="3">
         <v>15501544784</v>
@@ -1104,21 +1097,21 @@
         <v>9560255055</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="9">
+        <v>12</v>
+      </c>
+      <c r="G21" s="7">
         <v>590479841</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" s="3">
         <v>15501029811</v>
@@ -1126,15 +1119,15 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" s="3">
         <v>15501544787</v>
@@ -1143,21 +1136,21 @@
         <v>9311107208</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="9">
+        <v>12</v>
+      </c>
+      <c r="G23" s="7">
         <v>590479901</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D24" s="3">
         <v>15501544783</v>
@@ -1166,40 +1159,40 @@
         <v>9953595755</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" s="9">
+        <v>12</v>
+      </c>
+      <c r="G24" s="7">
         <v>590479821</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" s="3">
         <v>15501029810</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="9">
+      <c r="G25" s="7">
         <v>596559035</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D26" s="3">
         <v>15501544785</v>
@@ -1208,40 +1201,40 @@
         <v>9871207208</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="9">
+        <v>12</v>
+      </c>
+      <c r="G26" s="7">
         <v>590479862</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27" s="3">
         <v>15501029812</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
-      <c r="G27" s="9">
+      <c r="G27" s="7">
         <v>596560694</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D28" s="3">
         <v>15501544786</v>
@@ -1250,21 +1243,21 @@
         <v>9311207208</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="9">
+        <v>12</v>
+      </c>
+      <c r="G28" s="7">
         <v>590479883</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D29" s="3">
         <v>15501544788</v>
@@ -1273,21 +1266,21 @@
         <v>8800522020</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="9">
+        <v>12</v>
+      </c>
+      <c r="G29" s="7">
         <v>590479922</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D30" s="3">
         <v>15501077163</v>
@@ -1296,19 +1289,19 @@
         <v>9953595755</v>
       </c>
       <c r="F30" s="3"/>
-      <c r="G30" s="9">
+      <c r="G30" s="7">
         <v>592387856</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D31" s="3">
         <v>15501029775</v>
@@ -1317,133 +1310,133 @@
         <v>9953595755</v>
       </c>
       <c r="F31" s="3"/>
-      <c r="G31" s="9">
+      <c r="G31" s="7">
         <v>592387856</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D32" s="3">
         <v>159871207208</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="3"/>
-      <c r="G32" s="9" t="s">
+      <c r="G32" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
-        <v>32</v>
-      </c>
       <c r="B33" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D33" s="3">
         <v>159311207208</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="3"/>
-      <c r="G33" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G33" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D34" s="3">
         <v>159871897208</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="3"/>
-      <c r="G34" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G34" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D35" s="3">
         <v>918800522020</v>
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="3"/>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="B36" s="3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D36" s="3">
         <v>50100494729252</v>
       </c>
       <c r="E36" s="6"/>
       <c r="F36" s="3"/>
-      <c r="G36" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G36" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D37" s="3">
         <v>59108826833384</v>
       </c>
       <c r="E37" s="6"/>
       <c r="F37" s="3"/>
-      <c r="G37" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G37" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D38" s="3">
         <v>50100481253815</v>
@@ -1452,21 +1445,21 @@
         <v>9311207208</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G38" s="9">
+        <v>55</v>
+      </c>
+      <c r="G38" s="7">
         <v>182886542</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D39" s="3">
         <v>50100481260290</v>
@@ -1475,21 +1468,21 @@
         <v>8851100933</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G39" s="9">
+        <v>55</v>
+      </c>
+      <c r="G39" s="7">
         <v>182888497</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D40" s="3">
         <v>50100481685763</v>
@@ -1498,21 +1491,21 @@
         <v>9871207208</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G40" s="9">
+        <v>55</v>
+      </c>
+      <c r="G40" s="7">
         <v>176310062</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D41" s="3">
         <v>50100482018525</v>
@@ -1521,21 +1514,21 @@
         <v>9871207208</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G41" s="9">
+        <v>55</v>
+      </c>
+      <c r="G41" s="7">
         <v>183067405</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D42" s="3">
         <v>50100450138673</v>
@@ -1544,21 +1537,21 @@
         <v>9871207208</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G42" s="9">
+        <v>55</v>
+      </c>
+      <c r="G42" s="7">
         <v>176310062</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D43" s="3">
         <v>50100498462021</v>
@@ -1567,21 +1560,21 @@
         <v>9953595755</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G43" s="9">
+        <v>55</v>
+      </c>
+      <c r="G43" s="7">
         <v>176310063</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D44" s="3">
         <v>50100274037141</v>
@@ -1590,21 +1583,21 @@
         <v>9560255055</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G44" s="10">
+        <v>57</v>
+      </c>
+      <c r="G44" s="8">
         <v>128512511</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D45" s="3">
         <v>50100502634845</v>
@@ -1613,42 +1606,45 @@
         <v>9311107208</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G45" s="9">
+        <v>55</v>
+      </c>
+      <c r="G45" s="7">
         <v>188674001</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D46" s="3">
         <v>10591678294</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="D47" s="3">
         <v>925020009337222</v>
       </c>
+      <c r="G47" t="s">
+        <v>61</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>